<commit_message>
Validación de login si falla el código de validación en 1s
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>JEFATURA ZONAL DE JUNIN</v>
+        <v>JEFTURA ZONAL DE JUNIN</v>
       </c>
       <c r="C3" t="str">
         <v>31/03/2026</v>
@@ -480,7 +480,7 @@
         <v>INICIAL DE LICENCIA DE USO</v>
       </c>
       <c r="F3" t="str">
-        <v>46724112</v>
+        <v>77276891</v>
       </c>
       <c r="G3" t="str">
         <v>029042-0</v>
@@ -576,7 +576,7 @@
         <v>INICIAL DE LICENCIA DE USO</v>
       </c>
       <c r="F6" t="str">
-        <v>46724112</v>
+        <v>77276891</v>
       </c>
       <c r="G6" t="str">
         <v>029042-0</v>
@@ -608,7 +608,7 @@
         <v>INICIAL DE LICENCIA DE USO</v>
       </c>
       <c r="F7" t="str">
-        <v>46724112</v>
+        <v>77276891</v>
       </c>
       <c r="G7" t="str">
         <v>029042-0</v>
@@ -623,9 +623,14 @@
         <v>Pendiente</v>
       </c>
     </row>
+    <row r="11">
+      <c r="D11" t="str">
+        <v>s</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Logica de validacion de cupos 0 y campo de observaciones agregado
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,28 +430,31 @@
       <c r="J1" t="str">
         <v>estado</v>
       </c>
+      <c r="K1" t="str">
+        <v>observaciones</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>JEFATURA ZONAL DE JUNIN</v>
+        <v>LIMA</v>
       </c>
       <c r="C2" t="str">
-        <v>31/03/2026</v>
+        <v>31/3/26</v>
       </c>
       <c r="D2" t="str">
-        <v>10:00-10:15</v>
+        <v>12:30-12:45</v>
       </c>
       <c r="E2" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
+        <v>RENOVACIÓN DE LICENCIA DE USO</v>
       </c>
       <c r="F2" t="str">
-        <v>46724112</v>
+        <v>44136452</v>
       </c>
       <c r="G2" t="str">
-        <v>029042-0</v>
+        <v>052340-0</v>
       </c>
       <c r="H2" t="str">
         <v>CORTA</v>
@@ -494,28 +497,31 @@
       <c r="J3" t="str">
         <v>Pendiente</v>
       </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>JEFATURA ZONAL LAMBAYEQUE (EX-INTENDENCIA II NORTE)</v>
+        <v>JEFATURA ZONAL DE JUNIN</v>
       </c>
       <c r="C4" t="str">
-        <v>31/3/26</v>
+        <v>31/03/2026</v>
       </c>
       <c r="D4" t="str">
-        <v>08:30-08:45</v>
+        <v>10:00-10:15</v>
       </c>
       <c r="E4" t="str">
-        <v>RENOVACIÓN DE LICENCIA DE USO</v>
+        <v>INICIAL DE LICENCIA DE USO</v>
       </c>
       <c r="F4" t="str">
-        <v>77276891</v>
+        <v>46724112</v>
       </c>
       <c r="G4" t="str">
-        <v>090086-0</v>
+        <v>029042-0</v>
       </c>
       <c r="H4" t="str">
         <v>CORTA</v>
@@ -525,6 +531,9 @@
       </c>
       <c r="J4" t="str">
         <v>Pendiente</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -550,87 +559,26 @@
         <v>090086-0</v>
       </c>
       <c r="H5" t="str">
-        <v>LARGA</v>
+        <v>CORTA</v>
       </c>
       <c r="I5" t="str">
-        <v>ESCOPETA</v>
+        <v>REVOLVER</v>
       </c>
       <c r="J5" t="str">
         <v>Pendiente</v>
       </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>JEFTURA ZONAL DE JUNIN</v>
-      </c>
-      <c r="C6" t="str">
-        <v>31/03/2026</v>
-      </c>
-      <c r="D6" t="str">
-        <v>10:00-10:15</v>
-      </c>
-      <c r="E6" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
-      </c>
-      <c r="F6" t="str">
-        <v>77276891</v>
-      </c>
-      <c r="G6" t="str">
-        <v>029042-0</v>
-      </c>
-      <c r="H6" t="str">
-        <v>CORTA</v>
-      </c>
-      <c r="I6" t="str">
-        <v>REVOLVER</v>
-      </c>
-      <c r="J6" t="str">
-        <v>Pendiente</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>JEFTURA ZONAL DE JUNIN</v>
-      </c>
-      <c r="C7" t="str">
-        <v>31/03/2026</v>
-      </c>
-      <c r="D7" t="str">
-        <v>10:00-10:15</v>
-      </c>
-      <c r="E7" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
-      </c>
-      <c r="F7" t="str">
-        <v>77276891</v>
-      </c>
-      <c r="G7" t="str">
-        <v>029042-0</v>
-      </c>
-      <c r="H7" t="str">
-        <v>LARGA</v>
-      </c>
-      <c r="I7" t="str">
-        <v>ESCOPETA</v>
-      </c>
-      <c r="J7" t="str">
-        <v>Pendiente</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="D11" t="str">
-        <v>s</v>
+      <c r="K6" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flujo pulido hasta el final con validaciones pendientes pero funcional
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -513,7 +513,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -528,12 +528,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>12:45-13:00</t>
+          <t>10:30-10:45</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>24/03/2026</t>
+          <t>25/03/2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>No alcanzo cupo para horario 12:30-12:45</t>
+          <t>No alcanzo cupo para horario 10:30-10:45</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Selva</t>
+          <t>J &amp; V Resguardo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>24/03/2026</t>
+          <t>25/03/2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Documento vigilante no disponible para esta razón social/RUC. DNI=46724112 | RUC=Selva</t>
+          <t>Error en procesamiento: No se encontró Nro Solicitud con token '29042'. Opciones: ['Seleccione']</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Selva</t>
+          <t>J &amp; V Resguardo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>24/03/2026</t>
+          <t>25/03/2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>24/03/2026</t>
+          <t>25/03/2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">

</xml_diff>

<commit_message>
Flujo pulido con validaciones y capturación de logs estructurado, así mismo se corrigió el error de no duplicidad de observaciones en registros que son de un solo examen de tiro
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -710,7 +710,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Error en procesamiento: No se encontró Nro Solicitud con token '29042'. Opciones: ['Seleccione']</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>